<commit_message>
Mise à jour page Lambris
</commit_message>
<xml_diff>
--- a/prix/lambris.xlsx
+++ b/prix/lambris.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\lambris\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6E0D5E-A1AB-4E72-B3B7-CE390136D4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5695FF4E-335C-4787-BD41-E0D4453DAA65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11016" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
@@ -635,7 +635,7 @@
         <v>8</v>
       </c>
       <c r="F2" s="21">
-        <v>100.86900000000659</v>
+        <v>71.39200000000659</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>6</v>
@@ -681,7 +681,7 @@
         <v>10</v>
       </c>
       <c r="F4" s="21">
-        <v>78.721999999996953</v>
+        <v>32.041999999996946</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>19</v>
@@ -704,7 +704,7 @@
         <v>11</v>
       </c>
       <c r="F5" s="21">
-        <v>82.419000000000437</v>
+        <v>42.287000000000432</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>20</v>
@@ -727,7 +727,7 @@
         <v>12</v>
       </c>
       <c r="F6" s="21">
-        <v>93.057999999999993</v>
+        <v>69.795999999999992</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>21</v>

</xml_diff>